<commit_message>
Add chat Excel import, start/end dates, demo GIF, and kanban roadmap.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/plan_biokad_demo.xlsx
+++ b/examples/plan_biokad_demo.xlsx
@@ -9,15 +9,21 @@
   <sheets>
     <sheet name="План" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$5:$I$27</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'План'!$5:$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +31,66 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F766E"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001C2422"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="005C6B66"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00134E4A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001C2422"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="005C6B66"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F766E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F7F4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +98,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDD4C8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDD4C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDD4C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDD4C8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -122,6 +229,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="419100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,753 +550,953 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>R&amp;D планирование</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>План: Импортированный план (BIO-X demo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Экспорт: 28.07.2026 16:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>код</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>задача</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>описание</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>исполнитель</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>длительность</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>дата начала</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>дата конца</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>предшественники</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>родитель</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Аналитика и целеполагание</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Формирование целевого профиля препарата</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="F6" s="9" t="n">
+        <v>46231</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>46246</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>T1.1</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Анализ рынка и unmet need</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Обзор конкурентов и unmet medical need</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Петрова</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E7" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
+      <c r="F7" s="14" t="n">
+        <v>46231</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>46236</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>T1.2</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>TPP draft</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Целевой профиль продукта (TPP)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Петрова</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E8" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F8" s="14" t="n">
+        <v>46236</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>46241</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>T1.1</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>T1.3</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Kick-off R&amp;D</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Установочное совещание команд</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Сидоров</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E9" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F9" s="14" t="n">
+        <v>46241</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>46243</v>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>T1.2</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Доклинические исследования</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>In vitro / in vivo пакет</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="n">
+      <c r="D10" s="6" t="inlineStr"/>
+      <c r="E10" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F10" s="9" t="n">
+        <v>46246</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>T2.1</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>In vitro эффективность (demo Excel)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Скрининг активности [из sample xlsx]</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>In vitro эффективность</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Скрининг активности</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Иванов</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E11" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
+      <c r="F11" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>46256</v>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>T2.2</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Токсикология</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>Предварительная токсикология</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Иванов</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E12" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F12" s="14" t="n">
+        <v>46256</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>46270</v>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>T2.1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>T2.3</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>PK/PD модель</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Фармакокинетика / фармакодинамика</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Козлова</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E13" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F13" s="14" t="n">
+        <v>46256</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>T2.1</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>T2.4</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Отчёт доклиники</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Сводный отчёт для регуляторики</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Иванов</t>
         </is>
       </c>
-      <c r="E10" t="n">
+      <c r="E14" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F14" s="14" t="n">
+        <v>46270</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>T2.2,T2.3</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>CMC / производство</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Химия, производство и контроль</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
+      <c r="D15" s="6" t="inlineStr"/>
+      <c r="E15" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F15" s="9" t="n">
+        <v>46286</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>T3.1</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Процесс синтеза DS</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Разработка процесса субстанции</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Смирнов</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E16" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr">
+      <c r="F16" s="14" t="n">
+        <v>46286</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H16" s="10" t="inlineStr"/>
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>T3.2</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Аналитические методы</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Методы контроля качества</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Смирнов</t>
         </is>
       </c>
-      <c r="E13" t="n">
+      <c r="E17" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F17" s="14" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>T3.1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>T3.3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Pilot batch</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Пилотная партия</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Орлова</t>
         </is>
       </c>
-      <c r="E14" t="n">
+      <c r="E18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F18" s="14" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>T3.2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>T3.4</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Стабильность (ускор.)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Ускоренные исследования стабильности</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Орлова</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E19" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F19" s="14" t="n">
+        <v>46318</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>46332</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>T3.3</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Регуляторика</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Подготовка досье</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="n">
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F20" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>46346</v>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>P2,P3</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>T4.1</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>CTD Module 2/3 draft</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Черновик модулей CTD</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>Васильева</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E21" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="F21" s="14" t="n">
+        <v>46231</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>46243</v>
+      </c>
+      <c r="H21" s="10" t="inlineStr"/>
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>T4.2</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Gap analysis</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C22" s="12" t="inlineStr">
         <is>
           <t>Анализ пробелов досье</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>Васильева</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E22" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F22" s="14" t="n">
+        <v>46243</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>46248</v>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
         <is>
           <t>T4.1</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>T4.3</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Pre-IND briefing</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Материалы pre-IND</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Сидоров</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E23" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F23" s="14" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>46329</v>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>T4.2,T2.4</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="I23" s="10" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Клиника I (подготовка)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Подготовка к FIH</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F24" s="9" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>46366</v>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>T5.1</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Протокол FIH draft</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Черновик протокола фазы I</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Морозов</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E25" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
+      <c r="F25" s="14" t="n">
+        <v>46231</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>46241</v>
+      </c>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="10" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>T5.2</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>Выбор клинической базы</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>Отбор сайта исследования</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>Морозов</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E26" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F26" s="14" t="n">
+        <v>46241</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>46248</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
         <is>
           <t>T5.1</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="I26" s="10" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>T5.3</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Этика / ИРБ пакет</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Пакет для этического комитета</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Васильева</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E27" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F27" s="14" t="n">
+        <v>46241</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>46249</v>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
         <is>
           <t>T5.1</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="I27" s="10" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Подсказка: при импорте сохраните заголовки. Колонки «дата начала» / «дата конца» задают сроки; если их нет — даты считаются по длительности и предшественникам.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A5:I27"/>
+  <mergeCells count="4">
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A29:I29"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add VAX-B demo plan, hidden UI action log, and selective undo for the agent.
Log human plan mutations as agent-only [UI_ACTION] messages with inverse ops, harden mass-shift/delete rules, and refresh demo seed/docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/plan_biokad_demo.xlsx
+++ b/examples/plan_biokad_demo.xlsx
@@ -10,7 +10,7 @@
     <sheet name="План" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$5:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'План'!$A$5:$J$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'План'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -558,10 +558,11 @@
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -574,14 +575,14 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>План: Импортированный план (BIO-X demo)</t>
+          <t>План: Импортированный план (VAX-B demo)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Экспорт: 28.07.2026 16:15</t>
+          <t>Экспорт: 29.07.2026 13:03</t>
         </is>
       </c>
     </row>
@@ -595,6 +596,7 @@
       <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -624,20 +626,25 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
+          <t>% выполнения</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
           <t>дата начала</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>дата конца</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>предшественники</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>родитель</t>
         </is>
@@ -651,28 +658,31 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Аналитика и целеполагание</t>
+          <t>Discovery и целеполагание</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Формирование целевого профиля препарата</t>
+          <t>Эпидемиология, платформа и TPP вакцинного кандидата VAX-B</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr"/>
       <c r="E6" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>46231</v>
+        <v>20</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>46246</v>
-      </c>
-      <c r="H6" s="6" t="inlineStr"/>
+        <v>46232</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>46252</v>
+      </c>
       <c r="I6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7">
+      <c r="J6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>T1.1</t>
@@ -680,12 +690,12 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Анализ рынка и unmet need</t>
+          <t>Эпидемиология и unmet need</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Обзор конкурентов и unmet medical need</t>
+          <t>Оценка бремени заболевания и конкурентного ландшафта (РФ/ЕАЭС)</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -694,16 +704,19 @@
         </is>
       </c>
       <c r="E7" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>46231</v>
+        <v>6</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>46236</v>
-      </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr">
+        <v>46232</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>46238</v>
+      </c>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -717,12 +730,12 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>TPP draft</t>
+          <t>Выбор платформы вакцины</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>Целевой профиль продукта (TPP)</t>
+          <t>Субъединичная / вектор / иная платформа — решение Go</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -733,18 +746,21 @@
       <c r="E8" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="14" t="n">
-        <v>46236</v>
+      <c r="F8" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>46241</v>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
+        <v>46238</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>46243</v>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>T1.1</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -758,12 +774,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Kick-off R&amp;D</t>
+          <t>Дизайн антигена и TPP</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Установочное совещание команд</t>
+          <t>Целевой профиль продукта (TPP) и конструкция антигена</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -772,20 +788,23 @@
         </is>
       </c>
       <c r="E9" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>46241</v>
+        <v>7</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>46243</v>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="14" t="n">
+        <v>46250</v>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>T1.2</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -804,25 +823,28 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>In vitro / in vivo пакет</t>
+          <t>Иммуногенность и безопасность до КИ (упрощённый пакет)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr"/>
       <c r="E10" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="F10" s="9" t="n">
-        <v>46246</v>
+        <v>45</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
+        <v>46252</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>46297</v>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -832,30 +854,33 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>In vitro эффективность</t>
+          <t>Иммуногенность in vitro</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Скрининг активности</t>
+          <t>Клеточные модели, нейтрализация / ELISA</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Иванов</t>
+          <t>Козлова</t>
         </is>
       </c>
       <c r="E11" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>46246</v>
+        <v>8</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="H11" s="10" t="inlineStr"/>
-      <c r="I11" s="10" t="inlineStr">
+        <v>46232</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>46240</v>
+      </c>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -869,12 +894,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Токсикология</t>
+          <t>Иммуногенность in vivo</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Предварительная токсикология</t>
+          <t>Животные модели, титры антител</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -885,18 +910,21 @@
       <c r="E12" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="F12" s="14" t="n">
-        <v>46256</v>
+      <c r="F12" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+        <v>46252</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>46266</v>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>T2.1</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -910,12 +938,12 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>PK/PD модель</t>
+          <t>Токсикология и местная переносимость</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Фармакокинетика / фармакодинамика</t>
+          <t>Предварительный tox-пакет для допуска к КИ</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -924,20 +952,23 @@
         </is>
       </c>
       <c r="E13" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <v>46256</v>
+        <v>12</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>46266</v>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
+        <v>46252</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>T2.1</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
+      <c r="J13" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -951,12 +982,12 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Отчёт доклиники</t>
+          <t>Сводный отчёт доклиники</t>
         </is>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>Сводный отчёт для регуляторики</t>
+          <t>Пакет для регуляторной подачи на КИ</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -965,20 +996,23 @@
         </is>
       </c>
       <c r="E14" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="F14" s="14" t="n">
-        <v>46270</v>
+        <v>8</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>46277</v>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
+        <v>46266</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>46274</v>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>T2.2,T2.3</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="J14" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -992,30 +1026,33 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>CMC / производство</t>
+          <t>CMC / производство DS–DP</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Химия, производство и контроль</t>
+          <t>Разработка процесса субстанции и готовой формы</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr"/>
       <c r="E15" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F15" s="9" t="n">
-        <v>46286</v>
+        <v>50</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>46321</v>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
+        <v>46297</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>46347</v>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -1025,12 +1062,12 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Процесс синтеза DS</t>
+          <t>Банк клеток / посевной материал</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Разработка процесса субстанции</t>
+          <t>Master / working cell bank или эквивалент платформы</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1039,16 +1076,19 @@
         </is>
       </c>
       <c r="E16" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="F16" s="14" t="n">
-        <v>46286</v>
+        <v>10</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>46298</v>
-      </c>
-      <c r="H16" s="10" t="inlineStr"/>
-      <c r="I16" s="10" t="inlineStr">
+        <v>46232</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>46242</v>
+      </c>
+      <c r="I16" s="10" t="inlineStr"/>
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -1062,34 +1102,37 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Аналитические методы</t>
+          <t>Процесс DS (антиген)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Методы контроля качества</t>
+          <t>Разработка и масштаб процесса субстанции</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Смирнов</t>
+          <t>Иванов</t>
         </is>
       </c>
       <c r="E17" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F17" s="14" t="n">
-        <v>46298</v>
+        <v>12</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>46308</v>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
+        <v>46242</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>46254</v>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>T3.1</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr">
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -1103,12 +1146,12 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Pilot batch</t>
+          <t>Формулирование DP</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Пилотная партия</t>
+          <t>Готовая лекарственная форма, адъювант / буфер</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -1119,18 +1162,21 @@
       <c r="E18" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="F18" s="14" t="n">
-        <v>46308</v>
+      <c r="F18" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
+        <v>46254</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>46264</v>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>T3.2</t>
         </is>
       </c>
-      <c r="I18" s="10" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -1144,12 +1190,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Стабильность (ускор.)</t>
+          <t>Аналитика и спецификации</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Ускоренные исследования стабильности</t>
+          <t>Методы контроля качества DS/DP</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -1158,109 +1204,122 @@
         </is>
       </c>
       <c r="E19" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>T3.2</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>T3.5</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Пилотная партия и ускоренная стабильность</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Engineering / pilot batch + ускоренная стабильность</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Орлова</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="F19" s="14" t="n">
-        <v>46318</v>
-      </c>
-      <c r="G19" s="14" t="n">
-        <v>46332</v>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>T3.3</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr">
+      <c r="F20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>T3.3,T3.4</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Регуляторика</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Подготовка досье</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr"/>
-      <c r="E20" s="8" t="n">
-        <v>25</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>46321</v>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>46346</v>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Регуляторика: разрешение на КИ</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Подача в Минздрав РФ / подготовка досье на КИ</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
+      <c r="E21" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>46347</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>46377</v>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>P2,P3</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>T4.1</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>CTD Module 2/3 draft</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Черновик модулей CTD</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>Васильева</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="F21" s="14" t="n">
-        <v>46231</v>
-      </c>
-      <c r="G21" s="14" t="n">
-        <v>46243</v>
-      </c>
-      <c r="H21" s="10" t="inlineStr"/>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
+      <c r="J21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>T4.2</t>
+          <t>T4.1</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Gap analysis</t>
+          <t>Черновик досье на КИ</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Анализ пробелов досье</t>
+          <t>Модули качества, доклиники и клинического протокола</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -1269,20 +1328,19 @@
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <v>46243</v>
+        <v>12</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>46248</v>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>T4.1</t>
-        </is>
-      </c>
-      <c r="I22" s="10" t="inlineStr">
+        <v>46232</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="I22" s="10" t="inlineStr"/>
+      <c r="J22" s="10" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
@@ -1291,128 +1349,141 @@
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>T4.3</t>
+          <t>T4.2</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Pre-IND briefing</t>
+          <t>Подача в Минздрав на КИ</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Материалы pre-IND</t>
+          <t>Комплект документов на разрешение клинических исследований</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Сидоров</t>
+          <t>Васильева</t>
         </is>
       </c>
       <c r="E23" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="F23" s="14" t="n">
-        <v>46321</v>
+      <c r="F23" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>46329</v>
-      </c>
-      <c r="H23" s="10" t="inlineStr">
-        <is>
-          <t>T4.2,T2.4</t>
-        </is>
+        <v>46274</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>46282</v>
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
+          <t>T4.1,T2.4</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
           <t>P4</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>T4.3</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Ответы на запросы регулятора</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Закрытие замечаний до получения разрешения</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Сидоров</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>46347</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>46357</v>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>T4.2</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Клиника I (подготовка)</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Подготовка к FIH</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr"/>
-      <c r="E24" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>46346</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>46366</v>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Клинические исследования I–III</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>КИ в РФ: безопасность, иммуногенность, эффективность</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr"/>
+      <c r="E25" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>46377</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>46497</v>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Протокол FIH draft</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>Черновик протокола фазы I</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Морозов</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F25" s="14" t="n">
-        <v>46231</v>
-      </c>
-      <c r="G25" s="14" t="n">
-        <v>46241</v>
-      </c>
-      <c r="H25" s="10" t="inlineStr"/>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
+      <c r="J25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>T5.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Выбор клинической базы</t>
+          <t>Фаза I: протокол и старт</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Отбор сайта исследования</t>
+          <t>FIH / первая в человеке — протокол, этика, старт набора</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
@@ -1421,20 +1492,19 @@
         </is>
       </c>
       <c r="E26" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="F26" s="14" t="n">
-        <v>46241</v>
+        <v>14</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>46248</v>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
+        <v>46232</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I26" s="10" t="inlineStr"/>
+      <c r="J26" s="10" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
@@ -1443,58 +1513,565 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
+          <t>T5.2</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Фаза I: набор и CSR</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Набор, безопасность, краткий клинический отчёт</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Морозов</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>46266</v>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>T5.1</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
           <t>T5.3</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Этика / ИРБ пакет</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>Пакет для этического комитета</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Фаза II: протокол и набор</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Доза / схема, иммуногенность, расширение популяции</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Морозов</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>46266</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>46290</v>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>T5.2</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>T5.4</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Фаза II: анализ иммуногенности</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Промежуточный анализ и решение Go для фазы III</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Козлова</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>T5.3</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>T5.5</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Фаза III: протокол и набор</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Многоцентровое исследование эффективности (РФ)</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Морозов</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>46377</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>46407</v>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>T5.4</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>T5.6</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Фаза III: первичные эндпоинты и CSR</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Закрытие базы, анализ, сводный клинический отчёт</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Морозов</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F31" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>46407</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>46427</v>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>T5.5</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Регистрация (Минздрав / ГРЛС)</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Получение регистрационного удостоверения в РФ</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr"/>
+      <c r="E32" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>46497</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>46537</v>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>P5,P3</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>T6.1</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Подача РУ в Минздрав</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Регистрационное досье на вакцину VAX-B</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>Васильева</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="F27" s="14" t="n">
-        <v>46241</v>
-      </c>
-      <c r="G27" s="14" t="n">
-        <v>46249</v>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>T5.1</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="E33" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>46232</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="I33" s="10" t="inlineStr"/>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>T6.2</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Экспертиза и запросы</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Экспертиза качества/эффективности, ответы на запросы</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Васильева</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>46497</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>46515</v>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>T6.1,T5.6</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>T6.3</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>РУ и внесение в ГРЛС</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Получение РУ, внесение в государственный реестр</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Сидоров</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>46515</v>
+      </c>
+      <c r="H35" s="14" t="n">
+        <v>46525</v>
+      </c>
+      <c r="I35" s="10" t="inlineStr">
+        <is>
+          <t>T6.2</t>
+        </is>
+      </c>
+      <c r="J35" s="10" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Коммерческое производство</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Валидация, серийный выпуск и batch release</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>46537</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>46582</v>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>T7.1</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Валидация процесса (PPQ)</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Process performance qualification серийного процесса</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Смирнов</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="F37" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>46232</v>
+      </c>
+      <c r="H37" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="I37" s="10" t="inlineStr"/>
+      <c r="J37" s="10" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Серийный выпуск DS/DP</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Коммерческие серии субстанции и готовой формы</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Орлова</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>46262</v>
+      </c>
+      <c r="I38" s="10" t="inlineStr">
+        <is>
+          <t>T7.1</t>
+        </is>
+      </c>
+      <c r="J38" s="10" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>T7.3</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Fill&amp;finish и упаковка</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Розлив, маркировка, вторичная упаковка</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Орлова</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F39" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>46262</v>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>T7.2</t>
+        </is>
+      </c>
+      <c r="J39" s="10" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>Подсказка: при импорте сохраните заголовки. Колонки «дата начала» / «дата конца» задают сроки; если их нет — даты считаются по длительности и предшественникам.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I27"/>
+  <autoFilter ref="A5:J39"/>
   <mergeCells count="4">
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="A41:J41"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>